<commit_message>
Kreator Postman: poprawki po testach na zywo
Umowa wymaga OkresDo, stanowiska i wydzialu. Pakiet 33 scenariuszy z wynikami.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H918m5w9176yCaoTPWeKqE
</commit_message>
<xml_diff>
--- a/Integracja/Kreator-Postman/Scenariusze testowe.xlsx
+++ b/Integracja/Kreator-Postman/Scenariusze testowe.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Scenariusze" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Scenariusze!$A$1:$I$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Scenariusze!$A$1:$I$34</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -64,169 +64,262 @@
     <t>Success = true, wersje biblioteki i enova, nazwa bazy.</t>
   </si>
   <si>
+    <t>test 30.10.2026</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Success=true. Pomyślnie przygotwano stan usługi</t>
+  </si>
+  <si>
+    <t>M-01</t>
+  </si>
+  <si>
+    <t>2 Minimum danych</t>
+  </si>
+  <si>
+    <t>Kartoteka: imię i nazwisko</t>
+  </si>
+  <si>
+    <t>UpdateEmployee</t>
+  </si>
+  <si>
+    <t>Sukces: kartoteka bez umowy, kod nadany z numeratora.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik</t>
+  </si>
+  <si>
+    <t>M-02</t>
+  </si>
+  <si>
+    <t>Kartoteka: plus kod</t>
+  </si>
+  <si>
+    <t>Sukces: kartoteka z własnym kodem, bez umowy.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-M02</t>
+  </si>
+  <si>
+    <t>M-03</t>
+  </si>
+  <si>
+    <t>Umowa bez OkresDo</t>
+  </si>
+  <si>
+    <t>Błąd: etat musi mieć datę końca.</t>
+  </si>
+  <si>
+    <t>Success=false. Błędny zakres dat (1.11.2026..)</t>
+  </si>
+  <si>
+    <t>M-04</t>
+  </si>
+  <si>
+    <t>Umowa bez OkresOd</t>
+  </si>
+  <si>
+    <t>Błąd: wymagana data początku.</t>
+  </si>
+  <si>
+    <t>Success=false. Wartość pola "Etat.Data" jest wymagana Etat: Specjalista</t>
+  </si>
+  <si>
+    <t>M-05</t>
+  </si>
+  <si>
+    <t>Umowa bez stanowiska</t>
+  </si>
+  <si>
+    <t>Błąd: wymagane stanowisko.</t>
+  </si>
+  <si>
+    <t>Success=false. Wartość pola "Etat.Stanowisko" jest wymagana Etat:</t>
+  </si>
+  <si>
+    <t>M-06</t>
+  </si>
+  <si>
+    <t>Umowa bez wydziału</t>
+  </si>
+  <si>
+    <t>Błąd: wymagany wydział.</t>
+  </si>
+  <si>
+    <t>Success=false. Wartość pola "Etat.Jednostka organizacyjna" jest wymagana Etat: Specjalista</t>
+  </si>
+  <si>
+    <t>M-07</t>
+  </si>
+  <si>
+    <t>MINIMUM: umowa na czas określony</t>
+  </si>
+  <si>
+    <t>Sukces: tylko cztery pola umowy. Bez typu umowy i wymiaru serwer nadaje wartości domyślne.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-M07</t>
+  </si>
+  <si>
+    <t>M-08</t>
+  </si>
+  <si>
+    <t>MINIMUM: umowa na czas nieokreślony</t>
+  </si>
+  <si>
+    <t>Sukces: OkresDo = 9999-12-31 zapisuje się w bazie jako 2099-12-31.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-M08</t>
+  </si>
+  <si>
+    <t>M-09</t>
+  </si>
+  <si>
+    <t>Z danymi do ZUS i PIT</t>
+  </si>
+  <si>
+    <t>Sukces: pełniejsze dane osobowe.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-M09</t>
+  </si>
+  <si>
+    <t>Z-01</t>
+  </si>
+  <si>
+    <t>3 Zatrudnienie</t>
+  </si>
+  <si>
+    <t>Czas nieokreślony, pełny etat</t>
+  </si>
+  <si>
+    <t>Nowy pracownik, Etat od 2026-11-01 bez końca.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-Z01</t>
+  </si>
+  <si>
+    <t>Z-02</t>
+  </si>
+  <si>
+    <t>Czas określony</t>
+  </si>
+  <si>
+    <t>Etat 2026-11-01 do 2027-10-31, typ: na czas określony.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-Z02</t>
+  </si>
+  <si>
+    <t>Z-03</t>
+  </si>
+  <si>
+    <t>Okres próbny</t>
+  </si>
+  <si>
+    <t>Etat do 2027-01-31, typ: na okres próbny.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-Z03</t>
+  </si>
+  <si>
+    <t>Z-04</t>
+  </si>
+  <si>
+    <t>Pół etatu</t>
+  </si>
+  <si>
+    <t>Wymiar etatu 1/2.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-Z04</t>
+  </si>
+  <si>
+    <t>Z-05</t>
+  </si>
+  <si>
+    <t>Z adresem, kontaktem i rachunkiem</t>
+  </si>
+  <si>
+    <t>Adres, e-mail i rachunek w kartotece.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-Z05</t>
+  </si>
+  <si>
+    <t>Z-06</t>
+  </si>
+  <si>
+    <t>Z cechą (pole dodatkowe)</t>
+  </si>
+  <si>
+    <t>Cecha zapisana. Wymaga zmiennej cecha z nazwą cechy z dostępem przez WebAPI; bez niej błąd braku definicji.</t>
+  </si>
+  <si>
     <t>dokumentacja</t>
   </si>
   <si>
-    <t>D-02</t>
-  </si>
-  <si>
-    <t>Czy cechy mają dostęp przez API</t>
+    <t>BŁĄD</t>
+  </si>
+  <si>
+    <t>Success=false. W tabeli 'Pracownicy' nie znaleziono definicji cechy o nazwie 'UZUPELNIJ'.</t>
+  </si>
+  <si>
+    <t>P-01</t>
+  </si>
+  <si>
+    <t>4 Przedłużenie</t>
+  </si>
+  <si>
+    <t>Przedłużenie umowy określonej</t>
+  </si>
+  <si>
+    <t>Nowy zapis historii od 2027-11-01, koniec Etatu 2028-10-31. Wystarczy OkresDo.</t>
+  </si>
+  <si>
+    <t>Success=true. Nastąpiła aktualizacja kartoteki pracownika wg klucza Kod: API-Z02</t>
+  </si>
+  <si>
+    <t>P-02</t>
+  </si>
+  <si>
+    <t>Kontrola po przedłużeniu</t>
   </si>
   <si>
     <t>GetEmployee</t>
   </si>
   <si>
-    <t>Po Z-01: lista Features pokazuje cechy dostępne przez API.</t>
-  </si>
-  <si>
-    <t>M-01</t>
-  </si>
-  <si>
-    <t>2 Minimum danych</t>
-  </si>
-  <si>
-    <t>Tylko imię i nazwisko</t>
-  </si>
-  <si>
-    <t>UpdateEmployee</t>
-  </si>
-  <si>
-    <t>Ustalić: czy wystarcza minimum ze schematu.</t>
-  </si>
-  <si>
-    <t>hipoteza</t>
-  </si>
-  <si>
-    <t>M-02</t>
-  </si>
-  <si>
-    <t>Plus kod</t>
-  </si>
-  <si>
-    <t>Ustalić: czy powstaje kartoteka bez umowy.</t>
-  </si>
-  <si>
-    <t>M-03</t>
-  </si>
-  <si>
-    <t>Plus sam początek umowy</t>
-  </si>
-  <si>
-    <t>Ustalić: czy wymagany jest typ umowy i wymiar.</t>
-  </si>
-  <si>
-    <t>M-04</t>
-  </si>
-  <si>
-    <t>Plus typ umowy i wymiar</t>
-  </si>
-  <si>
-    <t>Ustalić: czy wymagane są stanowisko i wydział.</t>
-  </si>
-  <si>
-    <t>M-05</t>
-  </si>
-  <si>
-    <t>Plus stanowisko i wydział</t>
-  </si>
-  <si>
-    <t>Ustalić: czy to komplet dla umowy o pracę.</t>
-  </si>
-  <si>
-    <t>M-06</t>
-  </si>
-  <si>
-    <t>Plus dane do ZUS i PIT</t>
-  </si>
-  <si>
-    <t>Komplet: pracownik gotowy do naliczeń; porównać z kartoteką w enova.</t>
-  </si>
-  <si>
-    <t>Z-01</t>
-  </si>
-  <si>
-    <t>3 Zatrudnienie</t>
-  </si>
-  <si>
-    <t>Czas nieokreślony, pełny etat</t>
-  </si>
-  <si>
-    <t>Nowy pracownik, Etat od 2026-11-01 bez końca.</t>
-  </si>
-  <si>
-    <t>Z-02</t>
-  </si>
-  <si>
-    <t>Czas określony</t>
-  </si>
-  <si>
-    <t>Etat 2026-11-01 do 2027-10-31, typ: na czas określony.</t>
-  </si>
-  <si>
-    <t>Z-03</t>
-  </si>
-  <si>
-    <t>Okres próbny</t>
-  </si>
-  <si>
-    <t>Etat do 2027-01-31, typ: na okres próbny.</t>
-  </si>
-  <si>
-    <t>Z-04</t>
-  </si>
-  <si>
-    <t>Pół etatu</t>
-  </si>
-  <si>
-    <t>Wymiar etatu 1/2.</t>
-  </si>
-  <si>
-    <t>Z-05</t>
-  </si>
-  <si>
-    <t>Z adresem, kontaktem i rachunkiem</t>
-  </si>
-  <si>
-    <t>Adres, e-mail i rachunek w kartotece.</t>
-  </si>
-  <si>
-    <t>Z-06</t>
-  </si>
-  <si>
-    <t>Z cechą (pole dodatkowe)</t>
-  </si>
-  <si>
-    <t>Cecha zapisana. Wymaga wpisania nazwy cechy z włączonym dostępem przez API.</t>
-  </si>
-  <si>
-    <t>P-01</t>
-  </si>
-  <si>
-    <t>4 Przedłużenie</t>
-  </si>
-  <si>
-    <t>Przedłużenie umowy określonej</t>
-  </si>
-  <si>
-    <t>Ustalić: nowy zapis historii od 2027-11-01, koniec Etatu 2028-10-31.</t>
-  </si>
-  <si>
-    <t>P-02</t>
-  </si>
-  <si>
-    <t>Kontrola po przedłużeniu</t>
-  </si>
-  <si>
     <t>OkresDo = 2028-10-31.</t>
   </si>
   <si>
+    <t>Success=true. Pomyślny odczyt</t>
+  </si>
+  <si>
     <t>P-03</t>
   </si>
   <si>
     <t>Zamiana na czas nieokreślony</t>
   </si>
   <si>
-    <t>Ustalić: typ zmieniony, koniec Etatu pusty. Brak OkresDo może nie czyścić daty końca.</t>
+    <t>Typ zmieniony, OkresDo = 9999-12-31.</t>
+  </si>
+  <si>
+    <t>Success=true. Nastąpiła aktualizacja kartoteki pracownika wg klucza Kod: API-Z03</t>
+  </si>
+  <si>
+    <t>P-04</t>
+  </si>
+  <si>
+    <t>Nowa umowa po przerwie</t>
+  </si>
+  <si>
+    <t>Nowy zapis z nowym okresem umowy. Wcześniejsza umowa zostaje w historii.</t>
+  </si>
+  <si>
+    <t>Success=true. Nastąpiła aktualizacja kartoteki pracownika wg klucza Kod: API-Z04</t>
   </si>
   <si>
     <t>R-01</t>
@@ -238,7 +331,10 @@
     <t>Koniec umowy i Zwolniony</t>
   </si>
   <si>
-    <t>Ustalić: koniec Etatu 2027-03-31, status zwolnienia w enova.</t>
+    <t>Nowy zapis od 2027-03-31, koniec Etatu 2027-03-31. Przyczyna i kod zwolnienia zostają puste.</t>
+  </si>
+  <si>
+    <t>Success=true. Nastąpiła aktualizacja kartoteki pracownika wg klucza Kod: API-Z01</t>
   </si>
   <si>
     <t>R-02</t>
@@ -247,7 +343,7 @@
     <t>Kontrola po zwolnieniu</t>
   </si>
   <si>
-    <t>Zwolniony = true, OkresDo = 2027-03-31.</t>
+    <t>Zwolniony = true, OkresDo = 2027-03-31. Na wcześniejszą datę Zwolniony = false.</t>
   </si>
   <si>
     <t>R-03</t>
@@ -256,7 +352,7 @@
     <t>Zmiana adresu po zwolnieniu</t>
   </si>
   <si>
-    <t>Ustalić: zwolnienie NIE może zniknąć (w poprzednim dodatku WebAPI aktualizacja je cofała).</t>
+    <t>Zwolnienie zostaje w historii, ale nowy zapis po końcu umowy nie ma etatu.</t>
   </si>
   <si>
     <t>C-01</t>
@@ -271,13 +367,16 @@
     <t>Nowy zapis historii z nowym nazwiskiem.</t>
   </si>
   <si>
+    <t>Success=true. Nastąpiła aktualizacja kartoteki pracownika wg klucza Kod: API-Z05</t>
+  </si>
+  <si>
     <t>C-02</t>
   </si>
   <si>
     <t>Częściowa aktualizacja</t>
   </si>
   <si>
-    <t>Ustalić: e-mail zmieniony, a adres i rachunek z Z-05 zostają.</t>
+    <t>E-mail zmieniony od daty, adres i rachunek bez zmian.</t>
   </si>
   <si>
     <t>C-03</t>
@@ -286,7 +385,7 @@
     <t>Zmiana stanowiska i wymiaru od daty</t>
   </si>
   <si>
-    <t>Ustalić: nowy zapis historii od 2027-02-01, wymiar 3/4, okres Etatu bez zmian.</t>
+    <t>Nowy zapis od daty, okres Etatu bez zmian. Późniejsze zapisy nie są nadpisywane.</t>
   </si>
   <si>
     <t>C-04</t>
@@ -295,7 +394,7 @@
     <t>Zmiana bez znacznika Aktualizuj</t>
   </si>
   <si>
-    <t>Ustalić: czy zmiana nadpisuje bieżący zapis bez historii.</t>
+    <t>Nadpisuje bieżący zapis historii bez nowego wpisu.</t>
   </si>
   <si>
     <t>N-01</t>
@@ -310,6 +409,9 @@
     <t>Odrzucenie: nie znaleziono wydziału.</t>
   </si>
   <si>
+    <t>Success=false. Nie znaleziono Wydziału (Jednostki organizacyjnej) o kodzie: NIE-MA-TAKIEGO</t>
+  </si>
+  <si>
     <t>N-02</t>
   </si>
   <si>
@@ -319,6 +421,9 @@
     <t>Odrzucenie: nie znaleziono pracownika.</t>
   </si>
   <si>
+    <t>Success=false. Nie znaleziono pracownika o podanym kluczu: 'Kod: NIE-MA-TAKIEGO'</t>
+  </si>
+  <si>
     <t>N-03</t>
   </si>
   <si>
@@ -328,22 +433,43 @@
     <t>Odrzucenie: brak klucza pracownika.</t>
   </si>
   <si>
+    <t>Success=false. Nie wprowadzono żadnego klucza po który można wyszukać pracownika (Kod, ID lub Guid)</t>
+  </si>
+  <si>
     <t>N-04</t>
   </si>
   <si>
     <t>Cecha bez nazwy</t>
   </si>
   <si>
-    <t>Odrzucenie: cecha musi mieć nazwę.</t>
+    <t>Sukces: cecha bez nazwy jest pomijana bez ostrzeżenia.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-N04</t>
   </si>
   <si>
     <t>N-05</t>
   </si>
   <si>
-    <t>Cecha historyczna bez daty</t>
-  </si>
-  <si>
-    <t>Odrzucenie: cecha historyczna wymaga UpdateDate.</t>
+    <t>Nieistniejąca cecha</t>
+  </si>
+  <si>
+    <t>Odrzucenie: brak definicji cechy.</t>
+  </si>
+  <si>
+    <t>Success=false. W tabeli 'Pracownicy' nie znaleziono definicji cechy o nazwie 'NIE_MA_TAKIEJ_CECHY'.</t>
+  </si>
+  <si>
+    <t>N-06</t>
+  </si>
+  <si>
+    <t>Aktualizacja nieistniejącego kodu</t>
+  </si>
+  <si>
+    <t>RYZYKO: zamiast błędu powstaje nowy pracownik. Przed aktualizacją sprawdź Kod przez GetEmployee.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-LITEROWKA</t>
   </si>
 </sst>
 </file>
@@ -729,7 +855,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="30">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -748,568 +874,846 @@
       <c r="F2" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3">
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" ht="30">
       <c r="A3" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" ht="30">
+      <c r="A4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="C4" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" ht="30">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" ht="30">
       <c r="A6" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" ht="30">
       <c r="A7" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" ht="45">
       <c r="A8" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="9" ht="30">
       <c r="A9" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" ht="30">
       <c r="A10" s="2" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="11">
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" ht="30">
       <c r="A11" s="2" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="12">
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" ht="30">
       <c r="A12" s="2" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="13">
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" ht="30">
       <c r="A13" s="2" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="14">
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="14" ht="30">
       <c r="A14" s="2" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="15" ht="30">
       <c r="A15" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="C15" s="2" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="16" ht="30">
       <c r="A16" s="2" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" ht="45">
       <c r="A17" s="2" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>14</v>
+        <v>79</v>
+      </c>
+      <c r="G17" t="s">
+        <v>80</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="18" ht="30">
       <c r="A18" s="2" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="19" ht="30">
       <c r="A19" s="2" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>22</v>
+        <v>89</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="20" ht="30">
       <c r="A20" s="2" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="21" ht="30">
       <c r="A21" s="2" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="22" ht="30">
       <c r="A22" s="2" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="23">
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="23" ht="30">
       <c r="A23" s="2" t="s">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>84</v>
+        <v>106</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>22</v>
+        <v>89</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="24" ht="30">
       <c r="A24" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" ht="30">
+      <c r="A25" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="26" ht="30">
+      <c r="A26" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="27" ht="30">
+      <c r="A27" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="s">
+    </row>
+    <row r="28" ht="30">
+      <c r="A28" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="29" ht="45">
+      <c r="A29" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="30" ht="30">
+      <c r="A30" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="E30" s="2" t="s">
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="31" ht="45">
+      <c r="A31" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="32" ht="30">
+      <c r="A32" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="33" ht="45">
+      <c r="A33" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="34" ht="45">
+      <c r="A34" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>149</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I30"/>
+  <autoFilter ref="A1:I34"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Kreator Postman: Kod opcjonalny przy zatrudnieniu
Brak kodu lub kod spoza bazy zaklada nowa kartoteke, to dzialanie zamierzone.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H918m5w9176yCaoTPWeKqE
</commit_message>
<xml_diff>
--- a/Integracja/Kreator-Postman/Scenariusze testowe.xlsx
+++ b/Integracja/Kreator-Postman/Scenariusze testowe.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Scenariusze" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Scenariusze!$A$1:$I$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Scenariusze!$A$1:$I$35</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -187,6 +187,15 @@
     <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-M09</t>
   </si>
   <si>
+    <t>M-10</t>
+  </si>
+  <si>
+    <t>Umowa bez kodu</t>
+  </si>
+  <si>
+    <t>Sukces: nowa kartoteka, numer nadany zgodnie ze schematem.</t>
+  </si>
+  <si>
     <t>Z-01</t>
   </si>
   <si>
@@ -463,13 +472,13 @@
     <t>N-06</t>
   </si>
   <si>
-    <t>Aktualizacja nieistniejącego kodu</t>
-  </si>
-  <si>
-    <t>RYZYKO: zamiast błędu powstaje nowy pracownik. Przed aktualizacją sprawdź Kod przez GetEmployee.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-LITEROWKA</t>
+    <t>Kod spoza bazy</t>
+  </si>
+  <si>
+    <t>Sukces: kod spoza bazy zakłada nową kartotekę z kodem z żądania.</t>
+  </si>
+  <si>
+    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-NOWY</t>
   </si>
 </sst>
 </file>
@@ -1120,17 +1129,17 @@
         <v>55</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>58</v>
-      </c>
       <c r="F12" s="2" t="s">
         <v>14</v>
       </c>
@@ -1138,293 +1147,293 @@
         <v>15</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" ht="30">
       <c r="A13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="14" ht="30">
       <c r="A14" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G14" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="15" ht="30">
       <c r="A15" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G15" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="16" ht="30">
       <c r="A16" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" s="2" t="s">
+      <c r="F16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G16" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" s="2" t="s">
+    </row>
+    <row r="17" ht="30">
+      <c r="A17" s="2" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="17" ht="45">
-      <c r="A17" s="2" t="s">
+      <c r="B17" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E17" s="2" t="s">
+      <c r="F17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="F17" s="2" t="s">
+    </row>
+    <row r="18" ht="45">
+      <c r="A18" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="G17" t="s">
+      <c r="B18" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="D18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="18" ht="30">
-      <c r="A18" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="G18" t="s">
         <v>83</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G18" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="19" ht="30">
       <c r="A19" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="F19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G19" t="s">
-        <v>15</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="20" ht="30">
       <c r="A20" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C20" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E20" s="2" t="s">
+      <c r="F20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G20" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="21" ht="30">
       <c r="A21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" s="2" t="s">
+      <c r="F21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G21" t="s">
-        <v>15</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="22" ht="30">
       <c r="A22" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="D22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="F22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G22" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="23" ht="30">
       <c r="A23" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="E23" s="2" t="s">
+      <c r="F23" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G23" t="s">
-        <v>15</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="24" ht="30">
@@ -1432,13 +1441,13 @@
         <v>108</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>109</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>110</v>
@@ -1450,7 +1459,7 @@
         <v>15</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" ht="30">
@@ -1458,17 +1467,17 @@
         <v>111</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="D25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>114</v>
-      </c>
       <c r="F25" s="2" t="s">
         <v>14</v>
       </c>
@@ -1476,33 +1485,33 @@
         <v>15</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" ht="30">
       <c r="A26" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E26" s="2" t="s">
+      <c r="F26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G26" t="s">
-        <v>15</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="27" ht="30">
@@ -1510,7 +1519,7 @@
         <v>119</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>120</v>
@@ -1528,7 +1537,7 @@
         <v>15</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>86</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" ht="30">
@@ -1536,7 +1545,7 @@
         <v>122</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>123</v>
@@ -1554,166 +1563,192 @@
         <v>15</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="29" ht="45">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="29" ht="30">
       <c r="A29" s="2" t="s">
         <v>125</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E29" s="2" t="s">
+      <c r="F29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" ht="45">
+      <c r="A30" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="F29" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G29" t="s">
-        <v>15</v>
-      </c>
-      <c r="H29" s="2" t="s">
+      <c r="B30" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="30" ht="30">
-      <c r="A30" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="E30" s="2" t="s">
+      <c r="F30" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="F30" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G30" t="s">
-        <v>15</v>
-      </c>
-      <c r="H30" s="2" t="s">
+    </row>
+    <row r="31" ht="30">
+      <c r="A31" s="2" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="31" ht="45">
-      <c r="A31" s="2" t="s">
+      <c r="B31" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="C31" s="2" t="s">
+      <c r="D31" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="E31" s="2" t="s">
+      <c r="F31" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F31" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G31" t="s">
-        <v>15</v>
-      </c>
-      <c r="H31" s="2" t="s">
+    </row>
+    <row r="32" ht="45">
+      <c r="A32" s="2" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="32" ht="30">
-      <c r="A32" s="2" t="s">
+      <c r="B32" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E32" s="2" t="s">
+      <c r="F32" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="F32" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G32" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" s="2" t="s">
+    </row>
+    <row r="33" ht="30">
+      <c r="A33" s="2" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="33" ht="45">
-      <c r="A33" s="2" t="s">
+      <c r="B33" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="C33" s="2" t="s">
+      <c r="D33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E33" s="2" t="s">
+      <c r="F33" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G33" t="s">
-        <v>15</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="34" ht="45">
       <c r="A34" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="C34" s="2" t="s">
+      <c r="D34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E34" s="2" t="s">
+      <c r="F34" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="F34" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G34" t="s">
-        <v>15</v>
-      </c>
-      <c r="H34" s="2" t="s">
+    </row>
+    <row r="35" ht="30">
+      <c r="A35" s="2" t="s">
         <v>149</v>
       </c>
+      <c r="B35" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G35" t="s">
+        <v>15</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>152</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I34"/>
+  <autoFilter ref="A1:I35"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Kreator Postman: aktualizacja wymaga kodu, osobna zmiana rachunku
Rachunek bez Aktualizuj, imie i nazwisko tylko przy ich zmianie.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H918m5w9176yCaoTPWeKqE
</commit_message>
<xml_diff>
--- a/Integracja/Kreator-Postman/Scenariusze testowe.xlsx
+++ b/Integracja/Kreator-Postman/Scenariusze testowe.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Scenariusze" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Scenariusze!$A$1:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Scenariusze!$A$1:$I$36</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -403,7 +403,19 @@
     <t>Zmiana bez znacznika Aktualizuj</t>
   </si>
   <si>
-    <t>Nadpisuje bieżący zapis historii bez nowego wpisu.</t>
+    <t>Nie używać przy zmianie danych: nadpisuje bieżący zapis historii bez nowego wpisu.</t>
+  </si>
+  <si>
+    <t>Success=true przy ponowieniu. Dwie pierwsze próby: timeout SQL i błąd modyfikacji zapisu (przyczyna nieustalona).</t>
+  </si>
+  <si>
+    <t>C-05</t>
+  </si>
+  <si>
+    <t>Zmiana rachunku bankowego</t>
+  </si>
+  <si>
+    <t>Rachunek dopisany i główny, bez aktualizacji i bez zapisu historii. Poprzednie rachunki zostają.</t>
   </si>
   <si>
     <t>N-01</t>
@@ -1566,7 +1578,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="29" ht="30">
+    <row r="29" ht="45">
       <c r="A29" s="2" t="s">
         <v>125</v>
       </c>
@@ -1589,15 +1601,15 @@
         <v>15</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="30" ht="45">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="30" ht="30">
       <c r="A30" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>130</v>
@@ -1615,21 +1627,21 @@
         <v>15</v>
       </c>
       <c r="H30" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="31" ht="45">
+      <c r="A31" s="2" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="31" ht="30">
-      <c r="A31" s="2" t="s">
+      <c r="B31" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>129</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>134</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>135</v>
@@ -1644,12 +1656,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="32" ht="45">
+    <row r="32" ht="30">
       <c r="A32" s="2" t="s">
         <v>137</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>138</v>
@@ -1670,18 +1682,18 @@
         <v>140</v>
       </c>
     </row>
-    <row r="33" ht="30">
+    <row r="33" ht="45">
       <c r="A33" s="2" t="s">
         <v>141</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>142</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>143</v>
@@ -1696,12 +1708,12 @@
         <v>144</v>
       </c>
     </row>
-    <row r="34" ht="45">
+    <row r="34" ht="30">
       <c r="A34" s="2" t="s">
         <v>145</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>146</v>
@@ -1722,12 +1734,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="35" ht="30">
+    <row r="35" ht="45">
       <c r="A35" s="2" t="s">
         <v>149</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>150</v>
@@ -1748,7 +1760,33 @@
         <v>152</v>
       </c>
     </row>
+    <row r="36" ht="30">
+      <c r="A36" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I35"/>
+  <autoFilter ref="A1:I36"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Kreator Postman: przebudowa pod API dodatku klienta
UpsertEmployee i UpsertTermination, 47 scenariuszy z wynikami, scenariusze stanowisk.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H918m5w9176yCaoTPWeKqE
</commit_message>
<xml_diff>
--- a/Integracja/Kreator-Postman/Scenariusze testowe.xlsx
+++ b/Integracja/Kreator-Postman/Scenariusze testowe.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Scenariusze" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Scenariusze!$A$1:$I$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Scenariusze!$A$1:$I$48</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -73,63 +73,126 @@
     <t>Success=true. Pomyślnie przygotwano stan usługi</t>
   </si>
   <si>
+    <t>D-02</t>
+  </si>
+  <si>
+    <t>Dodatek odpowiada</t>
+  </si>
+  <si>
+    <t>GetOddzialy</t>
+  </si>
+  <si>
+    <t>Success = true, lista oddziałów.</t>
+  </si>
+  <si>
+    <t>Success=true. Pomyślnie odczytano paczkę rekordów z tabeli 'OddzialyFirmy'</t>
+  </si>
+  <si>
     <t>M-01</t>
   </si>
   <si>
     <t>2 Minimum danych</t>
   </si>
   <si>
-    <t>Kartoteka: imię i nazwisko</t>
-  </si>
-  <si>
-    <t>UpdateEmployee</t>
-  </si>
-  <si>
-    <t>Sukces: kartoteka bez umowy, kod nadany z numeratora.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik</t>
+    <t>MINIMUM: umowa na czas nieokreślony</t>
+  </si>
+  <si>
+    <t>UpsertEmployee</t>
+  </si>
+  <si>
+    <t>Sukces: imię, nazwisko i cztery pola umowy.</t>
+  </si>
+  <si>
+    <t>Success=true. Employee was successfully added/updated</t>
   </si>
   <si>
     <t>M-02</t>
   </si>
   <si>
-    <t>Kartoteka: plus kod</t>
-  </si>
-  <si>
-    <t>Sukces: kartoteka z własnym kodem, bez umowy.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-M02</t>
+    <t>MINIMUM: umowa na czas określony</t>
+  </si>
+  <si>
+    <t>Sukces: jak wyżej + data końca.</t>
   </si>
   <si>
     <t>M-03</t>
   </si>
   <si>
-    <t>Umowa bez OkresDo</t>
-  </si>
-  <si>
-    <t>Błąd: etat musi mieć datę końca.</t>
-  </si>
-  <si>
-    <t>Success=false. Błędny zakres dat (1.11.2026..)</t>
+    <t>Kartoteka bez umowy</t>
+  </si>
+  <si>
+    <t>Sukces: kartoteka bez zatrudnienia.</t>
   </si>
   <si>
     <t>M-04</t>
   </si>
   <si>
-    <t>Umowa bez OkresOd</t>
-  </si>
-  <si>
-    <t>Błąd: wymagana data początku.</t>
-  </si>
-  <si>
-    <t>Success=false. Wartość pola "Etat.Data" jest wymagana Etat: Specjalista</t>
+    <t>Bez kodu</t>
+  </si>
+  <si>
+    <t>Sukces: numer nadany zgodnie ze schematem.</t>
   </si>
   <si>
     <t>M-05</t>
   </si>
   <si>
+    <t>Z polami dodatkowymi</t>
+  </si>
+  <si>
+    <t>Sukces: wymaga cech Numer koncernowy i Typ pracownika.</t>
+  </si>
+  <si>
+    <t>M-06</t>
+  </si>
+  <si>
+    <t>Bez imienia</t>
+  </si>
+  <si>
+    <t>Błąd: wymagane imię.</t>
+  </si>
+  <si>
+    <t>Success=false. Wartość pola "Imie" jest wymagana PracHistoria: Testowy (K-M06), (wszystko)</t>
+  </si>
+  <si>
+    <t>M-07</t>
+  </si>
+  <si>
+    <t>Bez nazwiska</t>
+  </si>
+  <si>
+    <t>Błąd: wymagane nazwisko.</t>
+  </si>
+  <si>
+    <t>Success=false. Wartość pola "Nazwisko" jest wymagana PracHistoria: Jan (K-M07), (wszystko)</t>
+  </si>
+  <si>
+    <t>M-08</t>
+  </si>
+  <si>
+    <t>Umowa bez początku</t>
+  </si>
+  <si>
+    <t>Błąd: pole etatu tylko do odczytu, bo etat nie ma okresu.</t>
+  </si>
+  <si>
+    <t>Success=false. Próba zmiany wartości pola 'Etat.Jednostka organizacyjna' - pole w trybie 'tylko do odczytu' (Testowy Jan (K-M08), (wszystko))</t>
+  </si>
+  <si>
+    <t>M-09</t>
+  </si>
+  <si>
+    <t>Umowa bez typu</t>
+  </si>
+  <si>
+    <t>Błąd: wymagany typ umowy.</t>
+  </si>
+  <si>
+    <t>Success=false. Wymagane jest wprowadzenie wartości pola 'Etat.Typ umowy' (Testowy Jan (K-M09), (wszystko))</t>
+  </si>
+  <si>
+    <t>M-10</t>
+  </si>
+  <si>
     <t>Umowa bez stanowiska</t>
   </si>
   <si>
@@ -139,61 +202,16 @@
     <t>Success=false. Wartość pola "Etat.Stanowisko" jest wymagana Etat:</t>
   </si>
   <si>
-    <t>M-06</t>
+    <t>M-11</t>
   </si>
   <si>
     <t>Umowa bez wydziału</t>
   </si>
   <si>
-    <t>Błąd: wymagany wydział.</t>
-  </si>
-  <si>
-    <t>Success=false. Wartość pola "Etat.Jednostka organizacyjna" jest wymagana Etat: Specjalista</t>
-  </si>
-  <si>
-    <t>M-07</t>
-  </si>
-  <si>
-    <t>MINIMUM: umowa na czas określony</t>
-  </si>
-  <si>
-    <t>Sukces: tylko cztery pola umowy. Bez typu umowy i wymiaru serwer nadaje wartości domyślne.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-M07</t>
-  </si>
-  <si>
-    <t>M-08</t>
-  </si>
-  <si>
-    <t>MINIMUM: umowa na czas nieokreślony</t>
-  </si>
-  <si>
-    <t>Sukces: OkresDo = 9999-12-31 zapisuje się w bazie jako 2099-12-31.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-M08</t>
-  </si>
-  <si>
-    <t>M-09</t>
-  </si>
-  <si>
-    <t>Z danymi do ZUS i PIT</t>
-  </si>
-  <si>
-    <t>Sukces: pełniejsze dane osobowe.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-M09</t>
-  </si>
-  <si>
-    <t>M-10</t>
-  </si>
-  <si>
-    <t>Umowa bez kodu</t>
-  </si>
-  <si>
-    <t>Sukces: nowa kartoteka, numer nadany zgodnie ze schematem.</t>
+    <t>Błąd: pole etatu tylko do odczytu, bo etat nie ma wydziału.</t>
+  </si>
+  <si>
+    <t>Success=false. Próba zmiany wartości pola 'Etat.Definicja stanowiska' - pole w trybie 'tylko do odczytu' (Testowy Jan (K-M11), (wszystko))</t>
   </si>
   <si>
     <t>Z-01</t>
@@ -205,10 +223,7 @@
     <t>Czas nieokreślony, pełny etat</t>
   </si>
   <si>
-    <t>Nowy pracownik, Etat od 2026-11-01 bez końca.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-Z01</t>
+    <t>Nowy pracownik, etat bez końca.</t>
   </si>
   <si>
     <t>Z-02</t>
@@ -217,10 +232,7 @@
     <t>Czas określony</t>
   </si>
   <si>
-    <t>Etat 2026-11-01 do 2027-10-31, typ: na czas określony.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-Z02</t>
+    <t>Etat do 2027-10-31.</t>
   </si>
   <si>
     <t>Z-03</t>
@@ -232,19 +244,13 @@
     <t>Etat do 2027-01-31, typ: na okres próbny.</t>
   </si>
   <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-Z03</t>
-  </si>
-  <si>
     <t>Z-04</t>
   </si>
   <si>
     <t>Pół etatu</t>
   </si>
   <si>
-    <t>Wymiar etatu 1/2.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-Z04</t>
+    <t>Wymiar 1/2.</t>
   </si>
   <si>
     <t>Z-05</t>
@@ -253,28 +259,13 @@
     <t>Z adresem, kontaktem i rachunkiem</t>
   </si>
   <si>
-    <t>Adres, e-mail i rachunek w kartotece.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-Z05</t>
+    <t>Dane w kartotece, płeć wyliczona z PESEL.</t>
   </si>
   <si>
     <t>Z-06</t>
   </si>
   <si>
-    <t>Z cechą (pole dodatkowe)</t>
-  </si>
-  <si>
-    <t>Cecha zapisana. Podmień NAZWA_CECHY na cechę z dostępem przez WebAPI; bez niej błąd braku definicji.</t>
-  </si>
-  <si>
-    <t>dokumentacja</t>
-  </si>
-  <si>
-    <t>BŁĄD</t>
-  </si>
-  <si>
-    <t>Success=false. W tabeli 'Pracownicy' nie znaleziono definicji cechy o nazwie 'UZUPELNIJ'.</t>
+    <t>Cechy Numer koncernowy i Typ pracownika zapisane.</t>
   </si>
   <si>
     <t>P-01</t>
@@ -286,10 +277,7 @@
     <t>Przedłużenie umowy określonej</t>
   </si>
   <si>
-    <t>Nowy zapis historii od 2027-11-01, koniec Etatu 2028-10-31. Wystarczy OkresDo.</t>
-  </si>
-  <si>
-    <t>Success=true. Nastąpiła aktualizacja kartoteki pracownika wg klucza Kod: API-Z02</t>
+    <t>Nowy zapis historii od daty zmiany, koniec etatu 2028-10-31.</t>
   </si>
   <si>
     <t>P-02</t>
@@ -313,10 +301,7 @@
     <t>Zamiana na czas nieokreślony</t>
   </si>
   <si>
-    <t>Typ zmieniony, OkresDo = 9999-12-31.</t>
-  </si>
-  <si>
-    <t>Success=true. Nastąpiła aktualizacja kartoteki pracownika wg klucza Kod: API-Z03</t>
+    <t>Typ zmieniony, koniec etatu usunięty.</t>
   </si>
   <si>
     <t>P-04</t>
@@ -325,10 +310,22 @@
     <t>Nowa umowa po przerwie</t>
   </si>
   <si>
-    <t>Nowy zapis z nowym okresem umowy. Wcześniejsza umowa zostaje w historii.</t>
-  </si>
-  <si>
-    <t>Success=true. Nastąpiła aktualizacja kartoteki pracownika wg klucza Kod: API-Z04</t>
+    <t>Nowy okres umowy, wcześniejsza umowa zostaje w historii.</t>
+  </si>
+  <si>
+    <t>kod dodatku</t>
+  </si>
+  <si>
+    <t>P-05</t>
+  </si>
+  <si>
+    <t>Przedłużenie bez typu umowy</t>
+  </si>
+  <si>
+    <t>Błąd: każda aktualizacja umowy musi mieć typ.</t>
+  </si>
+  <si>
+    <t>Success=false. Wymagane jest wprowadzenie wartości pola 'Etat.Typ umowy' (Testowy Jan (K-Z02), 1.11.2028...)</t>
   </si>
   <si>
     <t>R-01</t>
@@ -337,13 +334,16 @@
     <t>5 Zwolnienie</t>
   </si>
   <si>
-    <t>Koniec umowy i Zwolniony</t>
-  </si>
-  <si>
-    <t>Nowy zapis od 2027-03-31, koniec Etatu 2027-03-31. Przyczyna i kod zwolnienia zostają puste.</t>
-  </si>
-  <si>
-    <t>Success=true. Nastąpiła aktualizacja kartoteki pracownika wg klucza Kod: API-Z01</t>
+    <t>Rozwiązanie umowy</t>
+  </si>
+  <si>
+    <t>UpsertTermination</t>
+  </si>
+  <si>
+    <t>Koniec etatu 2027-03-31, przyczyna zapisana.</t>
+  </si>
+  <si>
+    <t>Success=true. The employee's contract has been updated successfully</t>
   </si>
   <si>
     <t>R-02</t>
@@ -352,16 +352,34 @@
     <t>Kontrola po zwolnieniu</t>
   </si>
   <si>
-    <t>Zwolniony = true, OkresDo = 2027-03-31. Na wcześniejszą datę Zwolniony = false.</t>
+    <t>OkresDo = 2027-03-31.</t>
   </si>
   <si>
     <t>R-03</t>
   </si>
   <si>
+    <t>Przyczyna spoza słownika</t>
+  </si>
+  <si>
+    <t>RYZYKO: Success = true, a przyczyna zostaje pusta.</t>
+  </si>
+  <si>
+    <t>R-04</t>
+  </si>
+  <si>
     <t>Zmiana adresu po zwolnieniu</t>
   </si>
   <si>
-    <t>Zwolnienie zostaje w historii, ale nowy zapis po końcu umowy nie ma etatu.</t>
+    <t>Zwolnienie zostaje: żądanie nie ma sekcji Zatrudnienie.</t>
+  </si>
+  <si>
+    <t>R-05</t>
+  </si>
+  <si>
+    <t>Aktualizacja umowy cofa zwolnienie</t>
+  </si>
+  <si>
+    <t>RYZYKO: etat wraca do stanu bez końca, zwolnienie znika.</t>
   </si>
   <si>
     <t>C-01</t>
@@ -376,52 +394,127 @@
     <t>Nowy zapis historii z nowym nazwiskiem.</t>
   </si>
   <si>
-    <t>Success=true. Nastąpiła aktualizacja kartoteki pracownika wg klucza Kod: API-Z05</t>
-  </si>
-  <si>
     <t>C-02</t>
   </si>
   <si>
-    <t>Częściowa aktualizacja</t>
-  </si>
-  <si>
-    <t>E-mail zmieniony od daty, adres i rachunek bez zmian.</t>
+    <t>Zmiana e-maila</t>
+  </si>
+  <si>
+    <t>Nowy e-mail od daty zmiany.</t>
   </si>
   <si>
     <t>C-03</t>
   </si>
   <si>
-    <t>Zmiana stanowiska i wymiaru od daty</t>
-  </si>
-  <si>
-    <t>Nowy zapis od daty, okres Etatu bez zmian. Późniejsze zapisy nie są nadpisywane.</t>
+    <t>Zmiana adresu z województwem</t>
+  </si>
+  <si>
+    <t>Adres zmieniony, województwo zachowane.</t>
   </si>
   <si>
     <t>C-04</t>
   </si>
   <si>
-    <t>Zmiana bez znacznika Aktualizuj</t>
-  </si>
-  <si>
-    <t>Nie używać przy zmianie danych: nadpisuje bieżący zapis historii bez nowego wpisu.</t>
-  </si>
-  <si>
-    <t>Success=true przy ponowieniu. Dwie pierwsze próby: timeout SQL i błąd modyfikacji zapisu (przyczyna nieustalona).</t>
+    <t>Zmiana adresu bez województwa</t>
+  </si>
+  <si>
+    <t>RYZYKO: województwo zmienia się na nieokreślone.</t>
   </si>
   <si>
     <t>C-05</t>
   </si>
   <si>
-    <t>Zmiana rachunku bankowego</t>
-  </si>
-  <si>
-    <t>Rachunek dopisany i główny, bez aktualizacji i bez zapisu historii. Poprzednie rachunki zostają.</t>
+    <t>Zmiana rachunku</t>
+  </si>
+  <si>
+    <t>Rachunek dopisany i domyślny. Tworzy zapis historii.</t>
+  </si>
+  <si>
+    <t>C-06</t>
+  </si>
+  <si>
+    <t>Zmiana rachunku bez daty</t>
+  </si>
+  <si>
+    <t>Błąd: ta wersja dodatku wymaga DataAktualizacji przy każdej zmianie.</t>
+  </si>
+  <si>
+    <t>Success=false. No employee updated/added</t>
+  </si>
+  <si>
+    <t>C-07</t>
+  </si>
+  <si>
+    <t>Zmiana z datą wsteczną</t>
+  </si>
+  <si>
+    <t>RYZYKO: wymiar 1/2 przechodzi też na późniejsze zapisy historii.</t>
+  </si>
+  <si>
+    <t>C-08</t>
+  </si>
+  <si>
+    <t>Zmiana ograniczona datą końca</t>
+  </si>
+  <si>
+    <t>DataAktualizacji.To ogranicza zmianę: zapis od 2027-06-01 zostaje bez zmian.</t>
+  </si>
+  <si>
+    <t>S-01</t>
+  </si>
+  <si>
+    <t>7 Stanowiska</t>
+  </si>
+  <si>
+    <t>Zmiana stanowiska od daty</t>
+  </si>
+  <si>
+    <t>Definicja stanowiska zmieniona od daty, także w późniejszych zapisach. OkresDo musi być aktualny, inaczej zmiana cofa przedłużenie. Wymaga definicji Kierownik.</t>
+  </si>
+  <si>
+    <t>S-02</t>
+  </si>
+  <si>
+    <t>Kontrola stanowiska przed zmianą</t>
+  </si>
+  <si>
+    <t>Stanowisko = Specjalista.</t>
+  </si>
+  <si>
+    <t>S-03</t>
+  </si>
+  <si>
+    <t>Kontrola stanowiska po zmianie</t>
+  </si>
+  <si>
+    <t>Stanowisko = Kierownik.</t>
+  </si>
+  <si>
+    <t>S-04</t>
+  </si>
+  <si>
+    <t>Nieistniejąca definicja</t>
+  </si>
+  <si>
+    <t>Błąd: stanowisko musi istnieć w definicjach.</t>
+  </si>
+  <si>
+    <t>Success=false. Nie udało się pobrać definicji stanowiska o nazwie NIE-MA-TAKIEGO</t>
+  </si>
+  <si>
+    <t>S-05</t>
+  </si>
+  <si>
+    <t>Inna wielkość liter</t>
+  </si>
+  <si>
+    <t>Sukces: wyszukiwanie po nazwie nie rozróżnia wielkości liter.</t>
   </si>
   <si>
     <t>N-01</t>
   </si>
   <si>
-    <t>7 Błędy</t>
+    <t>8 Błędy</t>
   </si>
   <si>
     <t>Nieistniejący wydział</t>
@@ -430,7 +523,7 @@
     <t>Odrzucenie: nie znaleziono wydziału.</t>
   </si>
   <si>
-    <t>Success=false. Nie znaleziono Wydziału (Jednostki organizacyjnej) o kodzie: NIE-MA-TAKIEGO</t>
+    <t>Success=false. Nie udało się pobrać wydziału o kodzie NIE-MA-TAKIEGO</t>
   </si>
   <si>
     <t>N-02</t>
@@ -448,49 +541,31 @@
     <t>N-03</t>
   </si>
   <si>
-    <t>Odczyt bez klucza</t>
-  </si>
-  <si>
-    <t>Odrzucenie: brak klucza pracownika.</t>
-  </si>
-  <si>
-    <t>Success=false. Nie wprowadzono żadnego klucza po który można wyszukać pracownika (Kod, ID lub Guid)</t>
+    <t>Kod spoza bazy przy aktualizacji</t>
+  </si>
+  <si>
+    <t>Sukces: nowa kartoteka z kodem z żądania.</t>
   </si>
   <si>
     <t>N-04</t>
   </si>
   <si>
-    <t>Cecha bez nazwy</t>
-  </si>
-  <si>
-    <t>Sukces: cecha bez nazwy jest pomijana bez ostrzeżenia.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-N04</t>
+    <t>pars jako tablica</t>
+  </si>
+  <si>
+    <t>Wyjątek: ta wersja dodatku przyjmuje pojedynczy obiekt.</t>
+  </si>
+  <si>
+    <t>Success=undefined. The JSON value could not be converted to dodatek.Models.Dtos.EmployeeDTO. Path: $ | LineNumber: 0 | BytePositionInLine: 1.</t>
   </si>
   <si>
     <t>N-05</t>
   </si>
   <si>
-    <t>Nieistniejąca cecha</t>
-  </si>
-  <si>
-    <t>Odrzucenie: brak definicji cechy.</t>
-  </si>
-  <si>
-    <t>Success=false. W tabeli 'Pracownicy' nie znaleziono definicji cechy o nazwie 'NIE_MA_TAKIEJ_CECHY'.</t>
-  </si>
-  <si>
-    <t>N-06</t>
-  </si>
-  <si>
-    <t>Kod spoza bazy</t>
-  </si>
-  <si>
-    <t>Sukces: kod spoza bazy zakłada nową kartotekę z kodem z żądania.</t>
-  </si>
-  <si>
-    <t>Success=true. Do bazy danych został dodany nowy pracownik wg klucza Kod: API-NOWY</t>
+    <t>Zwolnienie nieistniejącego pracownika</t>
+  </si>
+  <si>
+    <t>Success=false. Employee code (PersonID) not found: NIE-MA-TAKIEGO</t>
   </si>
 </sst>
 </file>
@@ -907,42 +982,42 @@
         <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" ht="30">
       <c r="A4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>14</v>
@@ -951,24 +1026,24 @@
         <v>15</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" ht="30">
       <c r="A5" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>14</v>
@@ -977,7 +1052,7 @@
         <v>15</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" ht="30">
@@ -985,13 +1060,13 @@
         <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>32</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>33</v>
@@ -1003,233 +1078,233 @@
         <v>15</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" ht="30">
       <c r="A7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" ht="30">
+      <c r="A8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" s="2" t="s">
+      <c r="B8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="8" ht="45">
-      <c r="A8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="F8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" ht="45">
+      <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="2" t="s">
+      <c r="B9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="9" ht="30">
-      <c r="A9" s="2" t="s">
+      <c r="F9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="2" t="s">
+    </row>
+    <row r="10" ht="45">
+      <c r="A10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="10" ht="30">
-      <c r="A10" s="2" t="s">
+      <c r="F10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" s="2" t="s">
+    </row>
+    <row r="11" ht="60">
+      <c r="A11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="B11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="11" ht="30">
-      <c r="A11" s="2" t="s">
+      <c r="F11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="2" t="s">
+    </row>
+    <row r="12" ht="45">
+      <c r="A12" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="12" ht="30">
-      <c r="A12" s="2" t="s">
+      <c r="F12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="13" ht="30">
       <c r="A13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="F13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="2" t="s">
+    </row>
+    <row r="14" ht="60">
+      <c r="A14" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="B14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="14" ht="30">
-      <c r="A14" s="2" t="s">
+      <c r="F14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G14" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="15" ht="30">
       <c r="A15" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="F15" s="2" t="s">
         <v>14</v>
       </c>
@@ -1237,24 +1312,24 @@
         <v>15</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" ht="30">
       <c r="A16" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>14</v>
@@ -1263,76 +1338,76 @@
         <v>15</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>74</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" ht="30">
       <c r="A17" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" ht="30">
+      <c r="A18" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="D18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G17" t="s">
-        <v>15</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="18" ht="45">
-      <c r="A18" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="F18" s="2" t="s">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="G18" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>84</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" ht="30">
       <c r="A19" s="2" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>14</v>
@@ -1341,24 +1416,24 @@
         <v>15</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>89</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" ht="30">
       <c r="A20" s="2" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>91</v>
+        <v>38</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>92</v>
+        <v>25</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>14</v>
@@ -1367,24 +1442,24 @@
         <v>15</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>94</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" ht="30">
       <c r="A21" s="2" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>14</v>
@@ -1393,24 +1468,24 @@
         <v>15</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>98</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" ht="30">
       <c r="A22" s="2" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>14</v>
@@ -1419,24 +1494,24 @@
         <v>15</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23" ht="30">
       <c r="A23" s="2" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>14</v>
@@ -1445,50 +1520,50 @@
         <v>15</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>107</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" ht="30">
       <c r="A24" s="2" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>92</v>
+        <v>25</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="G24" t="s">
         <v>15</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="25" ht="30">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" ht="45">
       <c r="A25" s="2" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>14</v>
@@ -1497,50 +1572,50 @@
         <v>15</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" ht="30">
       <c r="A26" s="2" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="G26" t="s">
         <v>15</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" ht="30">
       <c r="A27" s="2" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>14</v>
@@ -1549,76 +1624,76 @@
         <v>15</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>118</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28" ht="30">
       <c r="A28" s="2" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="29" ht="30">
+      <c r="A29" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G28" t="s">
-        <v>15</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="29" ht="45">
-      <c r="A29" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>126</v>
-      </c>
       <c r="D29" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="G29" t="s">
         <v>15</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>128</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30" ht="30">
       <c r="A30" s="2" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>14</v>
@@ -1627,76 +1702,76 @@
         <v>15</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="31" ht="45">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" ht="30">
       <c r="A31" s="2" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="G31" t="s">
         <v>15</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>136</v>
+        <v>27</v>
       </c>
     </row>
     <row r="32" ht="30">
       <c r="A32" s="2" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>92</v>
+        <v>25</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="G32" t="s">
         <v>15</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="33" ht="45">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" ht="30">
       <c r="A33" s="2" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>92</v>
+        <v>25</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>14</v>
@@ -1705,50 +1780,50 @@
         <v>15</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>144</v>
+        <v>27</v>
       </c>
     </row>
     <row r="34" ht="30">
       <c r="A34" s="2" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35" ht="30">
+      <c r="A35" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G34" t="s">
-        <v>15</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="35" ht="45">
-      <c r="A35" s="2" t="s">
-        <v>149</v>
-      </c>
       <c r="B35" s="2" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>150</v>
+        <v>134</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>14</v>
@@ -1757,36 +1832,348 @@
         <v>15</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>152</v>
+        <v>27</v>
       </c>
     </row>
     <row r="36" ht="30">
       <c r="A36" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="37" ht="30">
+      <c r="A37" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="38" ht="30">
+      <c r="A38" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" t="s">
+        <v>15</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39" ht="45">
+      <c r="A39" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G39" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="40" ht="30">
+      <c r="A40" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G40" t="s">
+        <v>15</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="41" ht="30">
+      <c r="A41" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C36" s="2" t="s">
+      <c r="B41" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E36" s="2" t="s">
+      <c r="D41" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E41" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="F36" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G36" t="s">
-        <v>15</v>
-      </c>
-      <c r="H36" s="2" t="s">
+      <c r="F41" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="42" ht="30">
+      <c r="A42" s="2" t="s">
         <v>156</v>
       </c>
+      <c r="B42" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42" t="s">
+        <v>15</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="43" ht="30">
+      <c r="A43" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G43" t="s">
+        <v>15</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="44" ht="30">
+      <c r="A44" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44" t="s">
+        <v>15</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="45" ht="30">
+      <c r="A45" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G45" t="s">
+        <v>15</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="46" ht="30">
+      <c r="A46" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G46" t="s">
+        <v>15</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="47" ht="60">
+      <c r="A47" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G47" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="48" ht="30">
+      <c r="A48" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G48" t="s">
+        <v>15</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>181</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I36"/>
+  <autoFilter ref="A1:I48"/>
 </worksheet>
 </file>
</xml_diff>